<commit_message>
Tighten candidate priority and handoff reproducibility
</commit_message>
<xml_diff>
--- a/docs/audit_data/experimental_validation_handoff.xlsx
+++ b/docs/audit_data/experimental_validation_handoff.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1430b12c7219489f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate Panel" sheetId="2" r:id="R35c79b4382654001"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Result Entry" sheetId="3" r:id="R8772c3d206c441f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="4" r:id="Rabe87022997a4988"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="5" r:id="R52979fbd55a94ad3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R43280862ef724f24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidate Panel" sheetId="2" r:id="Rd88c0aa963c84871"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Result Entry" sheetId="3" r:id="Rc23be902065e46c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Log" sheetId="4" r:id="R762a8505b1464f7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="5" r:id="R69d54a3e465c423f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -812,7 +812,7 @@
         <x:color rgb="FF24543A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F3EC"/>
         </x:patternFill>
       </x:fill>
@@ -823,7 +823,7 @@
         <x:color rgb="FF9F2D25"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -1282,8 +1282,7 @@
         <x:v>Tier 2 candidates</x:v>
       </x:c>
       <x:c r="B9" s="46" t="n">
-        <x:f>COUNTIFS('Candidate Panel'!$E$6:$E$42,"Tier 2")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C9" s="36"/>
       <x:c r="D9" s="47" t="str">
@@ -1307,8 +1306,7 @@
         <x:v>Tier 3 candidates</x:v>
       </x:c>
       <x:c r="B10" s="46" t="n">
-        <x:f>COUNTIFS('Candidate Panel'!$E$6:$E$42,"Tier 3")</x:f>
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C10" s="36"/>
       <x:c r="D10" s="47" t="str">
@@ -1441,8 +1439,12 @@
       <x:c r="H18" s="58" t="str"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="36"/>
-      <x:c r="B19" s="36"/>
+      <x:c r="A19" s="36" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B19" s="36" t="str">
+        <x:v>Pareto membership alone does not determine priority; absolute CNS and specificity floors also apply.</x:v>
+      </x:c>
       <x:c r="C19" s="36"/>
       <x:c r="D19" s="36"/>
       <x:c r="E19" s="36"/>
@@ -1732,7 +1734,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S6" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>advance_if_stage_1_passes; prioritize by measured QC</x:v>
       </x:c>
       <x:c r="T6" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -1794,7 +1796,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S7" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>advance_if_stage_1_passes; prioritize by measured QC</x:v>
       </x:c>
       <x:c r="T7" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -1856,7 +1858,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S8" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>advance_if_stage_1_passes; prioritize by measured QC</x:v>
       </x:c>
       <x:c r="T8" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -1918,7 +1920,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S9" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>advance_if_stage_1_passes; prioritize by measured QC</x:v>
       </x:c>
       <x:c r="T9" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -1980,7 +1982,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S10" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>advance_if_stage_1_passes; prioritize by measured QC</x:v>
       </x:c>
       <x:c r="T10" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2042,7 +2044,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S11" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>advance_if_stage_1_passes; prioritize by measured QC</x:v>
       </x:c>
       <x:c r="T11" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2104,7 +2106,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S12" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>advance_if_stage_1_passes; prioritize by measured QC</x:v>
       </x:c>
       <x:c r="T12" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2133,7 +2135,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H13" s="80" t="str">
-        <x:v>strict_pareto_shortlist</x:v>
+        <x:v>target_plausible_pareto_shortlist</x:v>
       </x:c>
       <x:c r="I13" s="71" t="b">
         <x:v>0</x:v>
@@ -2166,7 +2168,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S13" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>advance_if_stage_1_passes; prioritize by measured QC</x:v>
       </x:c>
       <x:c r="T13" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2186,7 +2188,7 @@
         <x:v>computational_candidate</x:v>
       </x:c>
       <x:c r="E14" s="69" t="str">
-        <x:v>Tier 2</x:v>
+        <x:v>Tier 3</x:v>
       </x:c>
       <x:c r="F14" s="69" t="str">
         <x:v>low_liver</x:v>
@@ -2195,7 +2197,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="H14" s="80" t="str">
-        <x:v>strict_pareto_shortlist</x:v>
+        <x:v>exploratory_pareto_boundary_case</x:v>
       </x:c>
       <x:c r="I14" s="71" t="b">
         <x:v>0</x:v>
@@ -2228,7 +2230,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S14" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T14" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2290,7 +2292,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S15" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T15" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2352,7 +2354,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S16" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T16" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2414,7 +2416,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S17" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T17" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2476,7 +2478,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S18" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T18" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2538,7 +2540,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S19" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T19" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2600,7 +2602,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S20" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T20" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2662,7 +2664,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S21" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T21" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2724,7 +2726,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S22" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T22" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2786,7 +2788,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S23" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T23" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2848,7 +2850,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S24" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T24" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2910,7 +2912,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S25" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T25" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -2972,7 +2974,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S26" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T26" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -3034,7 +3036,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S27" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T27" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -3096,7 +3098,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S28" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T28" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -3158,7 +3160,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S29" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T29" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -3220,7 +3222,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S30" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T30" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -3282,7 +3284,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S31" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T31" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -3344,7 +3346,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S32" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T32" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -3406,7 +3408,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S33" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T33" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -3468,7 +3470,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S34" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T34" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -3530,7 +3532,7 @@
         <x:v>package_and_qc</x:v>
       </x:c>
       <x:c r="S35" s="80" t="str">
-        <x:v>advance_if_stage_1_passes</x:v>
+        <x:v>hold_after_stage_1; advance only by preregistered diversity challenge or measured QC</x:v>
       </x:c>
       <x:c r="T35" s="82" t="str">
         <x:v>rank_after_stage_2; test top 4-6</x:v>
@@ -3939,7 +3941,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9f814bf8b5e4ef7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R241ba56d0b3845c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8936,7 +8938,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5dfd81a4f164325"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad56dfd5ddce4ae1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10564,7 +10566,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0405148f5d2e4042"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R942aeb6890454040"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10994,7 +10996,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf295bd5c32f1419a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d96b9c9c3404f9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>